<commit_message>
sube pruebas en ltspice, y circuito svg para graficos
</commit_message>
<xml_diff>
--- a/hardware/Circuito Final/Switch banco - Torre/pines_entrada.xlsx
+++ b/hardware/Circuito Final/Switch banco - Torre/pines_entrada.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
@@ -9,13 +9,51 @@
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211" fullCalcOnLoad="1"/>
+  <calcPr calcId="122211"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
+  <si>
+    <t>VCC</t>
+  </si>
+  <si>
+    <t>DATA</t>
+  </si>
+  <si>
+    <t>LATCH</t>
+  </si>
+  <si>
+    <t>CLOCK</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>BUS NEG</t>
+  </si>
+  <si>
+    <t>BUS POS</t>
+  </si>
+  <si>
+    <t>BIT 2</t>
+  </si>
+  <si>
+    <t>BIT 1</t>
+  </si>
+  <si>
+    <t>SALIDA ADC</t>
+  </si>
+  <si>
+    <t>BIT 0</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,11 +90,19 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -98,7 +144,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -133,7 +179,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -341,10 +387,66 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="F4:L5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>2</v>
+      </c>
+      <c r="H5" t="s">
+        <v>4</v>
+      </c>
+      <c r="I5" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" t="s">
+        <v>6</v>
+      </c>
+      <c r="K5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>